<commit_message>
feat: integrate scheduling fairness and rule safeguards
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -17,6 +17,8 @@
     <sheet name="跨工作日资质预留" sheetId="12" r:id="rId12"/>
     <sheet name="末班重点航班范围" sheetId="13" r:id="rId13"/>
     <sheet name="跨航班重点岗位优先" sheetId="14" r:id="rId14"/>
+    <sheet name="末班重点次数修正" sheetId="15" r:id="rId15"/>
+    <sheet name="同航班人员互斥" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -423,18 +425,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1054,14 +1044,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1173,14 +1155,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1272,14 +1246,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1311,9 +1277,6 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1350,12 +1313,6 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1378,17 +1335,71 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>月份</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>人员编号</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>航班号</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>类别</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>修正次数</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>清零基准次数</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>规则ID</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>适用航班（空白表示全部）</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>人员A编号</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>人员A姓名</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>人员B编号</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>人员B姓名</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1500,13 +1511,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1603,10 +1607,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1682,16 +1682,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2742,13 +2732,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D26"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D27"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2962,161 +2946,175 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
-        <v>lateShiftRecoveryEnabled</v>
+        <v>tr121H02CooldownWorkdays</v>
       </c>
       <c r="B16" s="2" t="str">
-        <v>启用跨工作日恢复</v>
-      </c>
-      <c r="C16" s="2" t="str">
-        <v>是</v>
+        <v>TR121/H02 冷却工作班数</v>
+      </c>
+      <c r="C16" s="2">
+        <v>3</v>
       </c>
       <c r="D16" s="2" t="str">
-        <v>是否保护上一班末班重点岗位人员</v>
+        <v>承担 TR121/H02 后优先避开的后续已归档工作班数，0 表示关闭</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="str">
-        <v>nextWorkdayRecoveryMode</v>
+        <v>lateShiftRecoveryEnabled</v>
       </c>
       <c r="B17" s="2" t="str">
-        <v>跨工作日恢复目标强度</v>
+        <v>启用跨工作日恢复</v>
       </c>
       <c r="C17" s="2" t="str">
-        <v>prefer</v>
+        <v>是</v>
       </c>
       <c r="D17" s="2" t="str">
-        <v>优先避开或严格限制次班恢复目标</v>
+        <v>是否保护上一班末班重点岗位人员</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>lateShiftEndTime</v>
+        <v>nextWorkdayRecoveryMode</v>
       </c>
       <c r="B18" s="2" t="str">
-        <v>末班结束界线</v>
+        <v>跨工作日恢复目标强度</v>
       </c>
       <c r="C18" s="2" t="str">
-        <v>23:00</v>
+        <v>prefer</v>
       </c>
       <c r="D18" s="2" t="str">
-        <v>实际结束时间晚于该时刻的重点岗位纳入末班统计</v>
+        <v>优先避开或严格限制次班恢复目标</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>teamLeaderConcurrentSupervisionMaxOverlapMinutes</v>
+        <v>lateShiftEndTime</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>分队长并行督导最大重叠分钟</v>
-      </c>
-      <c r="C19" s="2">
-        <v>30</v>
+        <v>末班结束界线</v>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v>23:00</v>
       </c>
       <c r="D19" s="2" t="str">
-        <v>只在补齐常规岗位空缺时允许两个督导原始保障时段重叠的上限</v>
+        <v>实际结束时间晚于该时刻的重点岗位纳入末班统计</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>dutyFatiguePoints</v>
+        <v>teamLeaderConcurrentSupervisionMaxOverlapMinutes</v>
       </c>
       <c r="B20" s="2" t="str">
-        <v>值班疲劳点数</v>
+        <v>分队长并行督导最大重叠分钟</v>
       </c>
       <c r="C20" s="2">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D20" s="2" t="str">
-        <v>值班任务计入的疲劳点</v>
+        <v>只在补齐常规岗位空缺时允许两个督导原始保障时段重叠的上限</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
-        <v>earlyDepartureCutoffTime</v>
+        <v>dutyFatiguePoints</v>
       </c>
       <c r="B21" s="2" t="str">
-        <v>提前下班截载节点</v>
-      </c>
-      <c r="C21" s="2" t="str">
-        <v>12:00</v>
+        <v>值班疲劳点数</v>
+      </c>
+      <c r="C21" s="2">
+        <v>12</v>
       </c>
       <c r="D21" s="2" t="str">
-        <v>严格早于该时间计提前下班</v>
+        <v>值班任务计入的疲劳点</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="str">
-        <v>afternoonRestStartTime</v>
+        <v>earlyDepartureCutoffTime</v>
       </c>
       <c r="B22" s="2" t="str">
-        <v>下午无航班开始</v>
+        <v>提前下班截载节点</v>
       </c>
       <c r="C22" s="2" t="str">
         <v>12:00</v>
       </c>
       <c r="D22" s="2" t="str">
-        <v>下午无航班统计起点</v>
+        <v>严格早于该时间计提前下班</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="str">
-        <v>afternoonRestEndTime</v>
+        <v>afternoonRestStartTime</v>
       </c>
       <c r="B23" s="2" t="str">
-        <v>下午无航班结束</v>
+        <v>下午无航班开始</v>
       </c>
       <c r="C23" s="2" t="str">
-        <v>18:00</v>
+        <v>12:00</v>
       </c>
       <c r="D23" s="2" t="str">
-        <v>下午无航班统计终点</v>
+        <v>下午无航班统计起点</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="str">
-        <v>workloadBalanceEnabled</v>
+        <v>afternoonRestEndTime</v>
       </c>
       <c r="B24" s="2" t="str">
-        <v>启用工时疲劳均衡</v>
+        <v>下午无航班结束</v>
       </c>
       <c r="C24" s="2" t="str">
-        <v>是</v>
+        <v>18:00</v>
       </c>
       <c r="D24" s="2" t="str">
-        <v>是否执行人员负荷均衡</v>
+        <v>下午无航班统计终点</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="str">
-        <v>maxWorkHoursDifference</v>
+        <v>workloadBalanceEnabled</v>
       </c>
       <c r="B25" s="2" t="str">
-        <v>最大工时差</v>
-      </c>
-      <c r="C25" s="2">
-        <v>2</v>
+        <v>启用工时疲劳均衡</v>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v>是</v>
       </c>
       <c r="D25" s="2" t="str">
-        <v>常规人员当日工时差目标</v>
+        <v>是否执行人员负荷均衡</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="str">
+        <v>maxWorkHoursDifference</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v>最大工时差</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="str">
+        <v>常规人员当日工时差目标</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
         <v>maxTodayFatigueDifference</v>
       </c>
-      <c r="B26" s="2" t="str">
+      <c r="B27" s="2" t="str">
         <v>最大当日疲劳差</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C27" s="2">
         <v>4</v>
       </c>
-      <c r="D26" s="2" t="str">
+      <c r="D27" s="2" t="str">
         <v>常规人员当日疲劳差目标</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3124,17 +3122,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3204,12 +3191,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3263,12 +3244,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>

<commit_message>
feat(schedule): complete scheduling rule updates
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -16,9 +16,9 @@
     <sheet name="机动督导范围" sheetId="11" r:id="rId11"/>
     <sheet name="跨工作日资质预留" sheetId="12" r:id="rId12"/>
     <sheet name="末班重点航班范围" sheetId="13" r:id="rId13"/>
-    <sheet name="跨航班重点岗位优先" sheetId="14" r:id="rId14"/>
-    <sheet name="末班重点次数修正" sheetId="15" r:id="rId15"/>
-    <sheet name="同航班人员互斥" sheetId="16" r:id="rId16"/>
+    <sheet name="跨航班重点人员优先" sheetId="14" r:id="rId14"/>
+    <sheet name="同航班人员互斥" sheetId="15" r:id="rId15"/>
+    <sheet name="末班重点次数修正" sheetId="16" r:id="rId16"/>
   </sheets>
 </workbook>
 </file>
@@ -425,6 +425,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1044,6 +1056,14 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1155,6 +1175,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1246,6 +1274,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1277,6 +1313,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1312,7 +1351,14 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1325,12 +1371,15 @@
         <v>优先航班号</v>
       </c>
       <c r="D1" s="2" t="str">
-        <v>优先岗位（逗号分隔）</v>
+        <v>优先人员编号（逗号分隔）</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>优先人员姓名（仅供核对）</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1338,25 +1387,33 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
-        <v>月份</v>
+        <v>规则ID</v>
       </c>
       <c r="B1" s="2" t="str">
-        <v>人员编号</v>
+        <v>适用航班（空白表示全部）</v>
       </c>
       <c r="C1" s="2" t="str">
-        <v>航班号</v>
+        <v>人员A编号</v>
       </c>
       <c r="D1" s="2" t="str">
-        <v>类别</v>
+        <v>人员A姓名</v>
       </c>
       <c r="E1" s="2" t="str">
-        <v>修正次数</v>
+        <v>人员B编号</v>
       </c>
       <c r="F1" s="2" t="str">
-        <v>清零基准次数</v>
+        <v>人员B姓名</v>
       </c>
     </row>
   </sheetData>
@@ -1369,25 +1426,33 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
-        <v>规则ID</v>
+        <v>月份</v>
       </c>
       <c r="B1" s="2" t="str">
-        <v>适用航班（空白表示全部）</v>
+        <v>人员编号</v>
       </c>
       <c r="C1" s="2" t="str">
-        <v>人员A编号</v>
+        <v>航班号</v>
       </c>
       <c r="D1" s="2" t="str">
-        <v>人员A姓名</v>
+        <v>类别</v>
       </c>
       <c r="E1" s="2" t="str">
-        <v>人员B编号</v>
+        <v>修正次数</v>
       </c>
       <c r="F1" s="2" t="str">
-        <v>人员B姓名</v>
+        <v>清零基准次数</v>
       </c>
     </row>
   </sheetData>
@@ -1400,6 +1465,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1511,6 +1584,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1607,6 +1687,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1682,6 +1766,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2733,6 +2827,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3122,6 +3222,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3191,6 +3302,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3244,6 +3361,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>

<commit_message>
feat(schedule): add ordinary priority rotation
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -19,6 +19,8 @@
     <sheet name="跨航班重点人员优先" sheetId="14" r:id="rId14"/>
     <sheet name="同航班人员互斥" sheetId="15" r:id="rId15"/>
     <sheet name="末班重点次数修正" sheetId="16" r:id="rId16"/>
+    <sheet name="普通重点岗位集合" sheetId="17" r:id="rId17"/>
+    <sheet name="普通重点次数修正" sheetId="18" r:id="rId18"/>
   </sheets>
 </workbook>
 </file>
@@ -425,18 +427,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1056,14 +1046,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1175,14 +1157,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1274,14 +1248,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1313,9 +1279,6 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1352,13 +1315,6 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1387,14 +1343,6 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1426,14 +1374,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1447,6 +1387,144 @@
       </c>
       <c r="D1" s="2" t="str">
         <v>类别</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>修正次数</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>清零基准次数</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B12"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>航司</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>规范岗位</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>督导</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>G17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>G18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>G20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>FD</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>督导/引导</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>FD</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>G07</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>FD</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>G08</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>督导</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>H02</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>H04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>H05</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>月份</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>人员编号</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>航司</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>规范岗位</v>
       </c>
       <c r="E1" s="2" t="str">
         <v>修正次数</v>
@@ -1465,14 +1543,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1584,13 +1654,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1687,10 +1750,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1766,16 +1825,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2827,12 +2876,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3222,17 +3265,6 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3302,12 +3334,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3361,12 +3387,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>

<commit_message>
feat(schedule): expand coverage workflows
- add protected batch team-leader gap filling

- generalize mobile-supervisor fallback across flights

- preserve configuration, feedback, and safety contracts
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -8,19 +8,20 @@
     <sheet name="航班配置" sheetId="3" r:id="rId3"/>
     <sheet name="每周航班计划" sheetId="4" r:id="rId4"/>
     <sheet name="岗位配置" sheetId="5" r:id="rId5"/>
-    <sheet name="规则参数" sheetId="6" r:id="rId6"/>
-    <sheet name="岗位衔接规则" sheetId="7" r:id="rId7"/>
-    <sheet name="值班岗位优先" sheetId="8" r:id="rId8"/>
-    <sheet name="次班恢复目标" sheetId="9" r:id="rId9"/>
-    <sheet name="末班重点岗位" sheetId="10" r:id="rId10"/>
-    <sheet name="机动督导范围" sheetId="11" r:id="rId11"/>
-    <sheet name="跨工作日资质预留" sheetId="12" r:id="rId12"/>
-    <sheet name="末班重点航班范围" sheetId="13" r:id="rId13"/>
-    <sheet name="跨航班重点人员优先" sheetId="14" r:id="rId14"/>
-    <sheet name="同航班人员互斥" sheetId="15" r:id="rId15"/>
-    <sheet name="末班重点次数修正" sheetId="16" r:id="rId16"/>
-    <sheet name="普通重点岗位集合" sheetId="17" r:id="rId17"/>
-    <sheet name="普通重点次数修正" sheetId="18" r:id="rId18"/>
+    <sheet name="普通重点岗位集合" sheetId="6" r:id="rId6"/>
+    <sheet name="规则参数" sheetId="7" r:id="rId7"/>
+    <sheet name="岗位衔接规则" sheetId="8" r:id="rId8"/>
+    <sheet name="值班岗位优先" sheetId="9" r:id="rId9"/>
+    <sheet name="次班恢复目标" sheetId="10" r:id="rId10"/>
+    <sheet name="末班重点岗位" sheetId="11" r:id="rId11"/>
+    <sheet name="机动督导范围" sheetId="12" r:id="rId12"/>
+    <sheet name="跨工作日资质预留" sheetId="13" r:id="rId13"/>
+    <sheet name="末班重点航班范围" sheetId="14" r:id="rId14"/>
+    <sheet name="跨航班重点人员优先" sheetId="15" r:id="rId15"/>
+    <sheet name="同航班人员互斥" sheetId="16" r:id="rId16"/>
+    <sheet name="分队长补差保护范围" sheetId="17" r:id="rId17"/>
+    <sheet name="末班重点次数修正" sheetId="18" r:id="rId18"/>
+    <sheet name="普通重点次数修正" sheetId="19" r:id="rId19"/>
   </sheets>
 </workbook>
 </file>
@@ -427,6 +428,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1045,7 +1058,88 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D4"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>规则ID</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>航班号</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>岗位关键词</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>启用</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>recovery-target-cx937-one</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>CX937</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>一号</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>是</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>recovery-target-cx937-control</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>CX937</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>控制</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>是</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>recovery-target-ke166-one</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>KE166</v>
+      </c>
+      <c r="C4" s="2" t="str">
+        <v>一号</v>
+      </c>
+      <c r="D4" s="2" t="str">
+        <v>是</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1154,9 +1248,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1245,9 +1347,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1276,9 +1386,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1312,9 +1425,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1340,9 +1460,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1362,37 +1490,6 @@
       </c>
       <c r="F1" s="2" t="str">
         <v>人员B姓名</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="str">
-        <v>月份</v>
-      </c>
-      <c r="B1" s="2" t="str">
-        <v>人员编号</v>
-      </c>
-      <c r="C1" s="2" t="str">
-        <v>航班号</v>
-      </c>
-      <c r="D1" s="2" t="str">
-        <v>类别</v>
-      </c>
-      <c r="E1" s="2" t="str">
-        <v>修正次数</v>
-      </c>
-      <c r="F1" s="2" t="str">
-        <v>清零基准次数</v>
       </c>
     </row>
   </sheetData>
@@ -1404,107 +1501,27 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C1"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
-        <v>航司</v>
+        <v>航班号</v>
       </c>
       <c r="B1" s="2" t="str">
-        <v>规范岗位</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>CX</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>督导</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>CX</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>G17</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>CX</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>G18</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="str">
-        <v>CX</v>
-      </c>
-      <c r="B5" s="2" t="str">
-        <v>G20</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="str">
-        <v>FD</v>
-      </c>
-      <c r="B6" s="2" t="str">
-        <v>督导/引导</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="str">
-        <v>FD</v>
-      </c>
-      <c r="B7" s="2" t="str">
-        <v>G07</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="str">
-        <v>FD</v>
-      </c>
-      <c r="B8" s="2" t="str">
-        <v>G08</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="str">
-        <v>TR</v>
-      </c>
-      <c r="B9" s="2" t="str">
-        <v>督导</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="str">
-        <v>TR</v>
-      </c>
-      <c r="B10" s="2" t="str">
-        <v>H02</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="str">
-        <v>TR</v>
-      </c>
-      <c r="B11" s="2" t="str">
-        <v>H04</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="str">
-        <v>TR</v>
-      </c>
-      <c r="B12" s="2" t="str">
-        <v>H05</v>
+        <v>岗位名称</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>允许参与补差换人</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1512,6 +1529,53 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>月份</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>人员编号</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>航班号</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>类别</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>修正次数</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>清零基准次数</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1543,6 +1607,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1654,6 +1726,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1750,6 +1829,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1825,6 +1908,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2875,7 +2968,124 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>航司</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>规范岗位</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>督导</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>G17</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B4" s="2" t="str">
+        <v>G18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>CX</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>G20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="str">
+        <v>FD</v>
+      </c>
+      <c r="B6" s="2" t="str">
+        <v>督导/引导</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="str">
+        <v>FD</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>G07</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>FD</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>G08</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>督导</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>H02</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>H04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v>TR</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>H05</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D27"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3262,9 +3472,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3331,9 +3552,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3382,71 +3609,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="str">
-        <v>规则ID</v>
-      </c>
-      <c r="B1" s="2" t="str">
-        <v>航班号</v>
-      </c>
-      <c r="C1" s="2" t="str">
-        <v>岗位关键词</v>
-      </c>
-      <c r="D1" s="2" t="str">
-        <v>启用</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="str">
-        <v>recovery-target-cx937-one</v>
-      </c>
-      <c r="B2" s="2" t="str">
-        <v>CX937</v>
-      </c>
-      <c r="C2" s="2" t="str">
-        <v>一号</v>
-      </c>
-      <c r="D2" s="2" t="str">
-        <v>是</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="str">
-        <v>recovery-target-cx937-control</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>CX937</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>控制</v>
-      </c>
-      <c r="D3" s="2" t="str">
-        <v>是</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="str">
-        <v>recovery-target-ke166-one</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>KE166</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>一号</v>
-      </c>
-      <c r="D4" s="2" t="str">
-        <v>是</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D4"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: highlight manual schedule time conflicts
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -428,18 +428,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1059,12 +1047,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1132,14 +1114,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1251,14 +1225,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1350,14 +1316,6 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1389,9 +1347,6 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1428,13 +1383,6 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1463,14 +1411,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1502,11 +1442,6 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C1"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1529,14 +1464,6 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1568,14 +1495,6 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1607,14 +1526,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1726,13 +1637,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1829,10 +1733,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1908,16 +1808,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2969,10 +2859,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3079,13 +2965,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D27"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D28"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3299,175 +3179,189 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="str">
-        <v>tr121H02CooldownWorkdays</v>
+        <v>sameDayCrossFlightPriorityEnabled</v>
       </c>
       <c r="B16" s="2" t="str">
-        <v>TR121/H02 冷却工作班数</v>
-      </c>
-      <c r="C16" s="2">
-        <v>3</v>
+        <v>同日同航司控制/一号优先避免</v>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v>是</v>
       </c>
       <c r="D16" s="2" t="str">
-        <v>承担 TR121/H02 后优先避开的后续已归档工作班数，0 表示关闭</v>
+        <v>有安全替代时优先分开，无替代时允许安排并报警</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="str">
-        <v>lateShiftRecoveryEnabled</v>
+        <v>tr121H02CooldownWorkdays</v>
       </c>
       <c r="B17" s="2" t="str">
-        <v>启用跨工作日恢复</v>
-      </c>
-      <c r="C17" s="2" t="str">
-        <v>是</v>
+        <v>TR121/H02 冷却工作班数</v>
+      </c>
+      <c r="C17" s="2">
+        <v>3</v>
       </c>
       <c r="D17" s="2" t="str">
-        <v>是否保护上一班末班重点岗位人员</v>
+        <v>承担 TR121/H02 后优先避开的后续已归档工作班数，0 表示关闭</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="str">
-        <v>nextWorkdayRecoveryMode</v>
+        <v>lateShiftRecoveryEnabled</v>
       </c>
       <c r="B18" s="2" t="str">
-        <v>跨工作日恢复目标强度</v>
+        <v>启用跨工作日恢复</v>
       </c>
       <c r="C18" s="2" t="str">
-        <v>prefer</v>
+        <v>是</v>
       </c>
       <c r="D18" s="2" t="str">
-        <v>优先避开或严格限制次班恢复目标</v>
+        <v>是否保护上一班末班重点岗位人员</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="str">
-        <v>lateShiftEndTime</v>
+        <v>nextWorkdayRecoveryMode</v>
       </c>
       <c r="B19" s="2" t="str">
-        <v>末班结束界线</v>
+        <v>跨工作日恢复目标强度</v>
       </c>
       <c r="C19" s="2" t="str">
-        <v>23:00</v>
+        <v>prefer</v>
       </c>
       <c r="D19" s="2" t="str">
-        <v>实际结束时间晚于该时刻的重点岗位纳入末班统计</v>
+        <v>优先避开或严格限制次班恢复目标</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="str">
-        <v>teamLeaderConcurrentSupervisionMaxOverlapMinutes</v>
+        <v>lateShiftEndTime</v>
       </c>
       <c r="B20" s="2" t="str">
-        <v>分队长并行督导最大重叠分钟</v>
-      </c>
-      <c r="C20" s="2">
-        <v>30</v>
+        <v>末班结束界线</v>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v>23:00</v>
       </c>
       <c r="D20" s="2" t="str">
-        <v>只在补齐常规岗位空缺时允许两个督导原始保障时段重叠的上限</v>
+        <v>实际结束时间晚于该时刻的重点岗位纳入末班统计</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="str">
-        <v>dutyFatiguePoints</v>
+        <v>teamLeaderConcurrentSupervisionMaxOverlapMinutes</v>
       </c>
       <c r="B21" s="2" t="str">
-        <v>值班疲劳点数</v>
+        <v>分队长并行督导最大重叠分钟</v>
       </c>
       <c r="C21" s="2">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D21" s="2" t="str">
-        <v>值班任务计入的疲劳点</v>
+        <v>只在补齐常规岗位空缺时允许两个督导原始保障时段重叠的上限</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="str">
-        <v>earlyDepartureCutoffTime</v>
+        <v>dutyFatiguePoints</v>
       </c>
       <c r="B22" s="2" t="str">
-        <v>提前下班截载节点</v>
-      </c>
-      <c r="C22" s="2" t="str">
-        <v>12:00</v>
+        <v>值班疲劳点数</v>
+      </c>
+      <c r="C22" s="2">
+        <v>12</v>
       </c>
       <c r="D22" s="2" t="str">
-        <v>严格早于该时间计提前下班</v>
+        <v>值班任务计入的疲劳点</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="str">
-        <v>afternoonRestStartTime</v>
+        <v>earlyDepartureCutoffTime</v>
       </c>
       <c r="B23" s="2" t="str">
-        <v>下午无航班开始</v>
+        <v>提前下班截载节点</v>
       </c>
       <c r="C23" s="2" t="str">
         <v>12:00</v>
       </c>
       <c r="D23" s="2" t="str">
-        <v>下午无航班统计起点</v>
+        <v>严格早于该时间计提前下班</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="str">
-        <v>afternoonRestEndTime</v>
+        <v>afternoonRestStartTime</v>
       </c>
       <c r="B24" s="2" t="str">
-        <v>下午无航班结束</v>
+        <v>下午无航班开始</v>
       </c>
       <c r="C24" s="2" t="str">
-        <v>18:00</v>
+        <v>12:00</v>
       </c>
       <c r="D24" s="2" t="str">
-        <v>下午无航班统计终点</v>
+        <v>下午无航班统计起点</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="str">
-        <v>workloadBalanceEnabled</v>
+        <v>afternoonRestEndTime</v>
       </c>
       <c r="B25" s="2" t="str">
-        <v>启用工时疲劳均衡</v>
+        <v>下午无航班结束</v>
       </c>
       <c r="C25" s="2" t="str">
-        <v>是</v>
+        <v>18:00</v>
       </c>
       <c r="D25" s="2" t="str">
-        <v>是否执行人员负荷均衡</v>
+        <v>下午无航班统计终点</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="str">
-        <v>maxWorkHoursDifference</v>
+        <v>workloadBalanceEnabled</v>
       </c>
       <c r="B26" s="2" t="str">
-        <v>最大工时差</v>
-      </c>
-      <c r="C26" s="2">
-        <v>2</v>
+        <v>启用工时疲劳均衡</v>
+      </c>
+      <c r="C26" s="2" t="str">
+        <v>是</v>
       </c>
       <c r="D26" s="2" t="str">
-        <v>常规人员当日工时差目标</v>
+        <v>是否执行人员负荷均衡</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="str">
+        <v>maxWorkHoursDifference</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v>最大工时差</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2</v>
+      </c>
+      <c r="D27" s="2" t="str">
+        <v>常规人员当日工时差目标</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
         <v>maxTodayFatigueDifference</v>
       </c>
-      <c r="B27" s="2" t="str">
+      <c r="B28" s="2" t="str">
         <v>最大当日疲劳差</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C28" s="2">
         <v>4</v>
       </c>
-      <c r="D27" s="2" t="str">
+      <c r="D28" s="2" t="str">
         <v>常规人员当日疲劳差目标</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3475,17 +3369,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3555,12 +3438,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>

<commit_message>
feat: add configurable supervisor fill
- add guarded KE166 supervisor fill configuration and persistence
- align daily flight statistics and personnel conflict visibility
- tighten agent change authorization and sync rule documentation
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -15,13 +15,15 @@
     <sheet name="次班恢复目标" sheetId="10" r:id="rId10"/>
     <sheet name="末班重点岗位" sheetId="11" r:id="rId11"/>
     <sheet name="机动督导范围" sheetId="12" r:id="rId12"/>
-    <sheet name="跨工作日资质预留" sheetId="13" r:id="rId13"/>
-    <sheet name="末班重点航班范围" sheetId="14" r:id="rId14"/>
-    <sheet name="跨航班重点人员优先" sheetId="15" r:id="rId15"/>
-    <sheet name="同航班人员互斥" sheetId="16" r:id="rId16"/>
-    <sheet name="分队长补差保护范围" sheetId="17" r:id="rId17"/>
-    <sheet name="末班重点次数修正" sheetId="18" r:id="rId18"/>
-    <sheet name="普通重点次数修正" sheetId="19" r:id="rId19"/>
+    <sheet name="督导补位关系" sheetId="13" r:id="rId13"/>
+    <sheet name="跨工作日资质预留" sheetId="14" r:id="rId14"/>
+    <sheet name="末班重点航班范围" sheetId="15" r:id="rId15"/>
+    <sheet name="跨航班重点人员优先" sheetId="16" r:id="rId16"/>
+    <sheet name="同航班人员互斥" sheetId="17" r:id="rId17"/>
+    <sheet name="分队长补差保护范围" sheetId="18" r:id="rId18"/>
+    <sheet name="末班重点次数修正" sheetId="19" r:id="rId19"/>
+    <sheet name="普通重点次数修正" sheetId="20" r:id="rId20"/>
+    <sheet name="历史排班" sheetId="21" r:id="rId21"/>
   </sheets>
 </workbook>
 </file>
@@ -428,6 +430,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1047,6 +1061,12 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1114,6 +1134,14 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1225,6 +1253,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1315,7 +1351,88 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H2"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>规则ID</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>启用</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>来源航班</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>来源岗位关键词</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>目标航班</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>目标岗位关键词</v>
+      </c>
+      <c r="G1" s="2" t="str">
+        <v>允许自动补位</v>
+      </c>
+      <c r="H1" s="2" t="str">
+        <v>允许人工补位</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="str">
+        <v>ke166-h05-supervisor-fill</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>是</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>KE166</v>
+      </c>
+      <c r="D2" s="2" t="str">
+        <v>督导</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>KE166</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>H05</v>
+      </c>
+      <c r="G2" s="2" t="str">
+        <v>是</v>
+      </c>
+      <c r="H2" s="2" t="str">
+        <v>是</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1344,9 +1461,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1380,9 +1500,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1408,9 +1535,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1439,9 +1574,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C1"/>
+  <cols>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1461,9 +1601,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1477,37 +1625,6 @@
       </c>
       <c r="D1" s="2" t="str">
         <v>类别</v>
-      </c>
-      <c r="E1" s="2" t="str">
-        <v>修正次数</v>
-      </c>
-      <c r="F1" s="2" t="str">
-        <v>清零基准次数</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="str">
-        <v>月份</v>
-      </c>
-      <c r="B1" s="2" t="str">
-        <v>人员编号</v>
-      </c>
-      <c r="C1" s="2" t="str">
-        <v>航司</v>
-      </c>
-      <c r="D1" s="2" t="str">
-        <v>规范岗位</v>
       </c>
       <c r="E1" s="2" t="str">
         <v>修正次数</v>
@@ -1526,6 +1643,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1634,9 +1759,122 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>月份</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>人员编号</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>航司</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>规范岗位</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>修正次数</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>清零基准次数</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M1"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="32.83203125" customWidth="1"/>
+    <col min="12" max="12" width="20.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="str">
+        <v>记录ID</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <v>日期</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <v>航班号</v>
+      </c>
+      <c r="D1" s="2" t="str">
+        <v>岗位</v>
+      </c>
+      <c r="E1" s="2" t="str">
+        <v>人员编号</v>
+      </c>
+      <c r="F1" s="2" t="str">
+        <v>姓名</v>
+      </c>
+      <c r="G1" s="2" t="str">
+        <v>开始时间</v>
+      </c>
+      <c r="H1" s="2" t="str">
+        <v>结束时间</v>
+      </c>
+      <c r="I1" s="2" t="str">
+        <v>工作时长(小时)</v>
+      </c>
+      <c r="J1" s="2" t="str">
+        <v>疲劳点数</v>
+      </c>
+      <c r="K1" s="2" t="str">
+        <v>备注</v>
+      </c>
+      <c r="L1" s="2" t="str">
+        <v>历史覆盖范围</v>
+      </c>
+      <c r="M1" s="2" t="str">
+        <v>分队长补差</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1733,6 +1971,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1808,6 +2050,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2859,6 +3111,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2966,6 +3222,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D28"/>
+  <cols>
+    <col min="1" max="1" width="34.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3369,6 +3631,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3438,6 +3711,12 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>

<commit_message>
fix(balance): enforce daily flight count gap
Keep the deduplicated per-flight gap within one across all post-processing paths; leave structured vacancy evidence or reject the final result when balancing is unsafe.
</commit_message>
<xml_diff>
--- a/public/template/排班工具配置模板.xlsx
+++ b/public/template/排班工具配置模板.xlsx
@@ -430,18 +430,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J19"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1061,12 +1049,6 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D4"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1134,14 +1116,6 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1253,14 +1227,6 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1352,16 +1318,6 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H2"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1425,14 +1381,6 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1464,9 +1412,6 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A5"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1503,13 +1448,6 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1538,14 +1476,6 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1577,11 +1507,6 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C1"/>
-  <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1604,14 +1529,6 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1643,14 +1560,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1762,14 +1671,6 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F1"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1801,21 +1702,6 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M1"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="18.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="32.83203125" customWidth="1"/>
-    <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1868,13 +1754,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E5"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -1971,10 +1850,6 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="48.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -2050,16 +1925,6 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H40"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="48.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3111,10 +2976,6 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B12"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3221,13 +3082,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D28"/>
-  <cols>
-    <col min="1" max="1" width="34.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:D30"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3595,35 +3450,63 @@
     </row>
     <row r="27">
       <c r="A27" s="2" t="str">
-        <v>maxWorkHoursDifference</v>
+        <v>dailyFlightCountBalanceExemptHalfRest</v>
       </c>
       <c r="B27" s="2" t="str">
-        <v>最大工时差</v>
-      </c>
-      <c r="C27" s="2">
-        <v>2</v>
+        <v>半休人员豁免</v>
+      </c>
+      <c r="C27" s="2" t="str">
+        <v>是</v>
       </c>
       <c r="D27" s="2" t="str">
-        <v>常规人员当日工时差目标</v>
+        <v>勾选后半休人员不参与同一工作班航班数比较</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="str">
+        <v>dailyFlightCountBalanceExemptTeamLeaders</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>分队长豁免</v>
+      </c>
+      <c r="C28" s="2" t="str">
+        <v>是</v>
+      </c>
+      <c r="D28" s="2" t="str">
+        <v>勾选后分队长不参与同一工作班航班数比较</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>maxWorkHoursDifference</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>最大工时差</v>
+      </c>
+      <c r="C29" s="2">
+        <v>2</v>
+      </c>
+      <c r="D29" s="2" t="str">
+        <v>常规人员当日工时差目标</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
         <v>maxTodayFatigueDifference</v>
       </c>
-      <c r="B28" s="2" t="str">
+      <c r="B30" s="2" t="str">
         <v>最大当日疲劳差</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C30" s="2">
         <v>4</v>
       </c>
-      <c r="D28" s="2" t="str">
+      <c r="D30" s="2" t="str">
         <v>常规人员当日疲劳差目标</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D30"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -3631,17 +3514,6 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="14.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -3711,12 +3583,6 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D3"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">

</xml_diff>